<commit_message>
Add and complete all project backend APIs, production serving daemon, store, and machinery pages
</commit_message>
<xml_diff>
--- a/backend/login_data.xlsx
+++ b/backend/login_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
           <t>Password</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -459,6 +464,7 @@
           <t>password123</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -474,6 +480,7 @@
           <t>vbdevil</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -489,6 +496,7 @@
           <t>selvams</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -496,14 +504,551 @@
           <t>selvams</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>9025292383</t>
-        </is>
+      <c r="B5" t="n">
+        <v>9025292383</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>selvam</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9876543210</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>yasif</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bharan</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>9025292380</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Test Farmer</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9999999999</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tamil</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>9025292383</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>9998887771</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>9995180833</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>test_9995180833@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>9994561788</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>test_9994561788@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>9876500000</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>9995975712</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>test_9995975712@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>9994898238</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>test_9994898238@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9997837348</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>test_9997837348@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>9992210480</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>test_9992210480@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>9998117400</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>test_9998117400@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>9992681749</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>test_9992681749@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Real Test</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>9876543210</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>real@test.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>9993580759</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>test_9993580759@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>9998753124</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>test_9998753124@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>9992304155</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>test_9992304155@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>9993054221</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>test_9993054221@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>9992050563</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>test_9992050563@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>9999642000</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>test_9999642000@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>9997274501</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>test_9997274501@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>9991941138</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>test_9991941138@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>9998349533</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>test_9998349533@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>9991315478</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>test_9991315478@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>E2E Test User</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>9992526795</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>[HASHED]</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>test_9992526795@example.com</t>
         </is>
       </c>
     </row>

</xml_diff>